<commit_message>
feat(F-NAR-019): TREE-COL-021 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-021.xlsx
+++ b/stories/arbres/TREE-COL-021.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sous le portail, une flaque ronde tient le ciel. Le ciré jaune pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. Avec quoi commençons-nous ?</t>
+          <t>Sous le portail, une flaque ronde tient le ciel. Le ciré jaune pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. On commence avec quoi ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le portail, une flaque ronde tient le ciel. Le &lt;emphasis level="moderate"&gt;ciré jaune&lt;/emphasis&gt; pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. Avec quoi commençons-nous ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le portail, une flaque ronde tient le ciel. Le &lt;emphasis level="moderate"&gt;ciré jaune&lt;/emphasis&gt; pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. On commence avec quoi ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sous le portail, une flaque ronde tient le ciel. Le &lt;emphasis&gt;ciré jaune&lt;/emphasis&gt; pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. Avec quoi commençons-nous ? [pause]</t>
+          <t>Sous le portail, une flaque ronde tient le ciel. Le &lt;emphasis&gt;ciré jaune&lt;/emphasis&gt; pend au crochet. Le capuchon lourd laisse une goutte. La goutte tombe près des bottes. Ça sent le cacao, près de la vitre. La vapeur dessine un nuage sur le verre. Papa pose deux tasses tièdes. Maman cherche un gant sur le radiateur. Un merle parle, derrière le portail. En ce moment, Victorino tire le ciré. Je veux la flaque ! Le ciel est dedans ! Papa parle du cacao, à maman. Les mots se cognent aux tasses. Tu disais, Victorino ? La flaque, le ciel ! Papa écoute maman, pas lui. Victorino ferme la bouche. Il attend, près du crochet. Le cacao fait un petit nuage. Voilà, je t'écoute. Je veux aller à la flaque. On commence avec quoi ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
 narrateur|Le cacao fait un petit nuage.
 papa|Voilà, je t'écoute.
 enfant-m|Je veux aller à la flaque.
-maman|Avec quoi commençons-nous ?</t>
+maman|On commence avec quoi ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1395,17 +1395,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino peut prendre le ciré, les bottes, ou le bateau. Que prends-tu pour la flaque ?</t>
+          <t>Victorino peut prendre le ciré, les bottes, ou le bateau. Tu prends quoi, pour la flaque ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino peut prendre le ciré, les bottes, ou le bateau. Que prends-tu pour la flaque ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino peut prendre le ciré, les bottes, ou le bateau. Tu prends quoi, pour la flaque ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Victorino peut prendre le ciré, les bottes, ou le bateau. Que prends-tu pour la flaque ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Victorino peut prendre le ciré, les bottes, ou le bateau. Tu prends quoi, pour la flaque ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1564,7 +1564,7 @@
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Victorino peut prendre le ciré, les bottes, ou le bateau.
-maman|Que prends-tu pour la flaque ?</t>
+maman|Tu prends quoi, pour la flaque ?</t>
         </is>
       </c>
     </row>
@@ -1789,12 +1789,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Quelque chose tombe du capuchon. Qu'est-ce qui tombe ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Quelque chose tombe du &lt;emphasis level="moderate"&gt;capuchon&lt;/emphasis&gt;. Qu'est-ce qui tombe ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;soft&gt;&lt;slow&gt;Quelque chose tombe du capuchon. Qu'est-ce qui tombe ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Quelque chose tombe du &lt;emphasis&gt;capuchon&lt;/emphasis&gt;. Qu'est-ce qui tombe ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>goutte</t>
+          <t>capuchon</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
@@ -1977,12 +1977,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; ! Oui, une goutte du capuchon. Cette fois, papa a entendu. Merci, Victorino. Nous t'avons entendu. Le ciré craque, un peu collant. Une feuille jaune colle à la poche. Ils avancent vers la porte.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte ! Oui, une goutte du capuchon. Cette fois, papa a entendu. Merci, Victorino. Nous t'avons entendu. Le &lt;emphasis level="moderate"&gt;ciré&lt;/emphasis&gt; craque, un peu collant. Une feuille jaune colle à la poche. Ils avancent vers la porte.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Une &lt;emphasis&gt;goutte&lt;/emphasis&gt; ! Oui, une goutte du capuchon. Cette fois, papa a entendu. Merci, Victorino. Nous t'avons entendu. Le ciré craque, un peu collant. Une feuille jaune colle à la poche. Ils avancent vers la porte. [pause]</t>
+          <t>Une goutte ! Oui, une goutte du capuchon. Cette fois, papa a entendu. Merci, Victorino. Nous t'avons entendu. Le &lt;emphasis&gt;ciré&lt;/emphasis&gt; craque, un peu collant. Une feuille jaune colle à la poche. Ils avancent vers la porte. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>goutte</t>
+          <t>ciré</t>
         </is>
       </c>
       <c r="AI6" s="2" t="n">
@@ -2150,17 +2150,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?</t>
+          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
         <is>
           <t>narrateur|Dehors, l'eau brille en trois endroits.
 papa|La flaque du portail, la gouttière, ou le bac ?
-maman|Où allons-nous ?</t>
+maman|On va où ?</t>
         </is>
       </c>
     </row>
@@ -6431,17 +6431,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac.</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une goutte reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac. [pause]</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le ciré jaune sèche au soleil du bac. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6577,6 +6577,7 @@
         <is>
           <t>narrateur|Victorino choisit de regarder.
 narrateur|Papa garde les mains loin de l'arrosoir.
+narrateur|Une goutte reste au bec de l'arrosoir.
 maman|Il avance vers toi, Victorino.
 narrateur|Victorino ne répond pas.
 narrateur|Il laisse le silence au bateau.
@@ -6796,17 +6797,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Victorino attrape les bottes vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Les bottes font un petit ploc.</t>
+          <t>Victorino attrape les bottes vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Elles font ploc.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino attrape les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Les bottes font un petit ploc.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino attrape les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Elles font ploc.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Victorino attrape les &lt;emphasis&gt;bottes&lt;/emphasis&gt; vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Les bottes font un petit ploc. [pause]</t>
+          <t>Victorino attrape les &lt;emphasis&gt;bottes&lt;/emphasis&gt; vertes. Une botte est tiède, l'autre froide. Mes bottes, pour la flaque ! Maman cherche le gant, près du radiateur. Elle parle à papa du gant perdu. Les mots de Victorino tombent par terre. Maman ! Maman ne se tourne pas. Victorino pose une botte. Il attend, une chaussette à la main. Oui, je t'écoute. Il manque une chaussette. Elle chauffe, sur le radiateur. Maman tend la chaussette chaude. Victorino enfile le coton tiède. Elles font ploc. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6955,7 +6956,7 @@
 papa|Elle chauffe, sur le radiateur.
 narrateur|Maman tend la chaussette chaude.
 narrateur|Victorino enfile le coton tiède.
-papa|Les bottes font un petit ploc.</t>
+papa|Elles font ploc.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -6987,17 +6988,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Une botte attend son coton. Que manque-t-il, pour la botte ?</t>
+          <t>Une botte attend son coton. Il manque quoi, pour la botte ?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Une botte attend son coton. Que manque-t-il, pour la botte ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Une &lt;emphasis level="moderate"&gt;botte&lt;/emphasis&gt; attend son coton. Il manque quoi, pour la botte ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>&lt;soft&gt;&lt;slow&gt;Une botte attend son coton. Que manque-t-il, pour la botte ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Une &lt;emphasis&gt;botte&lt;/emphasis&gt; attend son coton. Il manque quoi, pour la botte ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -7094,7 +7095,7 @@
       </c>
       <c r="AH33" s="2" t="inlineStr">
         <is>
-          <t>chaussette</t>
+          <t>botte</t>
         </is>
       </c>
       <c r="AI33" s="2" t="n">
@@ -7148,7 +7149,7 @@
       <c r="AW33" t="inlineStr">
         <is>
           <t>narrateur|Une botte attend son coton.
-maman|Que manque-t-il, pour la botte ?</t>
+maman|Il manque quoi, pour la botte ?</t>
         </is>
       </c>
     </row>
@@ -7175,17 +7176,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>La chaussette ! Oui, la chaussette du radiateur. Maman l'a entendue, cette fois. Merci, Victorino. Tes mots sont arrivés. Les bottes font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu.</t>
+          <t>La chaussette ! Oui, la chaussette du radiateur. Maman a entendu, cette fois. Merci, Victorino. Tes mots sont arrivés. Les bottes font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chaussette&lt;/emphasis&gt; ! Oui, la chaussette du radiateur. Maman l'a entendue, cette fois. Merci, Victorino. Tes mots sont arrivés. Les bottes font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La chaussette ! Oui, la chaussette du radiateur. Maman a entendu, cette fois. Merci, Victorino. Tes mots sont arrivés. Les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chaussette&lt;/emphasis&gt; ! Oui, la chaussette du radiateur. Maman l'a entendue, cette fois. Merci, Victorino. Tes mots sont arrivés. Les bottes font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu. [pause]</t>
+          <t>La chaussette ! Oui, la chaussette du radiateur. Maman a entendu, cette fois. Merci, Victorino. Tes mots sont arrivés. Les &lt;emphasis&gt;bottes&lt;/emphasis&gt; font un petit ploc. Une feuille colle à la botte. La porte s'ouvre un peu. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7266,7 +7267,7 @@
       </c>
       <c r="AH34" s="2" t="inlineStr">
         <is>
-          <t>chaussette</t>
+          <t>bottes</t>
         </is>
       </c>
       <c r="AI34" s="2" t="n">
@@ -7321,7 +7322,7 @@
         <is>
           <t>enfant-m|La chaussette !
 narrateur|Oui, la chaussette du radiateur.
-narrateur|Maman l'a entendue, cette fois.
+narrateur|Maman a entendu, cette fois.
 papa|Merci, Victorino.
 papa|Tes mots sont arrivés.
 narrateur|Les bottes font un petit ploc.
@@ -7353,17 +7354,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?</t>
+          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -7523,7 +7524,7 @@
         <is>
           <t>narrateur|Dehors, l'eau brille en trois endroits.
 papa|La flaque du portail, la gouttière, ou le bac ?
-maman|Où allons-nous ?</t>
+maman|On va où ?</t>
         </is>
       </c>
     </row>
@@ -11634,17 +11635,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme.</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une goutte reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme. [pause]</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Une botte reflète le bac calme. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11780,6 +11781,7 @@
         <is>
           <t>narrateur|Victorino choisit de regarder.
 narrateur|Papa garde les mains loin de l'arrosoir.
+narrateur|Une goutte reste au bec de l'arrosoir.
 maman|Il avance vers toi, Victorino.
 narrateur|Victorino ne répond pas.
 narrateur|Il laisse le silence au bateau.
@@ -12190,17 +12192,17 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Victorino a un plan, pour l'eau. Que veut-il poser sur la flaque ?</t>
+          <t>Victorino a un plan, pour l'eau. Il veut poser quoi, sur la flaque ?</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino a un plan, pour l'eau. Que veut-il poser sur la flaque ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino a un plan, pour l'eau. Il veut poser quoi, sur la &lt;emphasis level="moderate"&gt;flaque&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>&lt;soft&gt;&lt;slow&gt;Victorino a un plan, pour l'eau. Que veut-il poser sur la flaque ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino a un plan, pour l'eau. Il veut poser quoi, sur la &lt;emphasis&gt;flaque&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -12297,7 +12299,7 @@
       </c>
       <c r="AH61" s="2" t="inlineStr">
         <is>
-          <t>bateau</t>
+          <t>flaque</t>
         </is>
       </c>
       <c r="AI61" s="2" t="n">
@@ -12351,7 +12353,7 @@
       <c r="AW61" t="inlineStr">
         <is>
           <t>narrateur|Victorino a un plan, pour l'eau.
-papa|Que veut-il poser sur la flaque ?</t>
+papa|Il veut poser quoi, sur la flaque ?</t>
         </is>
       </c>
     </row>
@@ -12556,17 +12558,17 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?</t>
+          <t>Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? Où allons-nous ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Dehors, l'eau brille en trois endroits. La flaque du portail, la gouttière, ou le bac ? On va où ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -12726,7 +12728,7 @@
         <is>
           <t>narrateur|Dehors, l'eau brille en trois endroits.
 papa|La flaque du portail, la gouttière, ou le bac ?
-maman|Où allons-nous ?</t>
+maman|On va où ?</t>
         </is>
       </c>
     </row>
@@ -16837,17 +16839,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille.</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une goutte reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille. [pause]</t>
+          <t>Victorino choisit de regarder. Papa garde les mains loin de l'arrosoir. Une &lt;emphasis&gt;goutte&lt;/emphasis&gt; reste au bec de l'arrosoir. Il avance vers toi, Victorino. Victorino ne répond pas. Il laisse le silence au bateau. Maintenant, tu peux poser l'arrosoir. Papa attend que le papier touche l'herbe. Le bateau sèche, plat comme une feuille. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -16983,6 +16985,7 @@
         <is>
           <t>narrateur|Victorino choisit de regarder.
 narrateur|Papa garde les mains loin de l'arrosoir.
+narrateur|Une goutte reste au bec de l'arrosoir.
 maman|Il avance vers toi, Victorino.
 narrateur|Victorino ne répond pas.
 narrateur|Il laisse le silence au bateau.
@@ -17196,7 +17199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17253,6 +17256,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>